<commit_message>
Uodate SRS Document C4
</commit_message>
<xml_diff>
--- a/SRS.xlsx
+++ b/SRS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SW Testing-iti 9m\Online-Mobile-Store-WebSite\Requirments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\GitFlow-C4-Alex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{648EC5FF-8C10-48BA-8C3A-1411BD0D8E05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781F0415-067B-4FD4-BA5E-6ABD2EBB045A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -467,7 +467,7 @@
     <t>The user shall be able to enter a username, email address, password, confirm password, address, phone number, National ID and User Type.</t>
   </si>
   <si>
-    <t>The username shall contain only alphabetic characters (a-z, A-Z)..</t>
+    <t>The username shall contain only alphabetic characters (a-z, A-Z)…</t>
   </si>
 </sst>
 </file>

</xml_diff>